<commit_message>
2026 09 15 001
1. 주석추가.
- 비상정지후 게속작업.
- buffer overflow 오류시 z축 상승.
- 대상트레이 z축 하강시 구간별 속도 변경.
</commit_message>
<xml_diff>
--- a/.IBC_인도 NGSORTER 셋업(2026 06).xlsx
+++ b/.IBC_인도 NGSORTER 셋업(2026 06).xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCE174E0-EFA5-43BD-829F-465BA1A577E7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84F46ADC-6439-4E8B-9FE6-4BADAA0F02B7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="8910" windowHeight="10470" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="656" uniqueCount="646">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="670" uniqueCount="655">
   <si>
     <t>내용</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -2035,7 +2035,7 @@
   <si>
     <r>
       <t xml:space="preserve">1. FMS 오류는 수동 조그 인터락에서 제외
-2. Source Centering 공통 인터락 제거
+2. Source Centering 공통 인터락 제거. source tray에서는 확인, target tray에서는 제거.
 </t>
     </r>
     <r>
@@ -2086,6 +2086,40 @@
       </rPr>
       <t>. (z축 이동시 센터링)</t>
     </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>fms alarm 시 설비에서 알람 on, 설비 알람 off시 fms alarm off.</t>
+  </si>
+  <si>
+    <t>tray info 요청한 시간 표시.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>수동일때 tray out 신호 off</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ems 버튼 불안들어옴.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>서보 무빙이 일정시간 지나면 servo moving 없애기.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>9/11</t>
+  </si>
+  <si>
+    <t>9/11</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>불량선별기 PLC 비상정지 버튼 눌렀을때 서보 멈춤. 에러표시 (pause, 알람)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>비상정지시 셀을 들고 있는 상태에서 홈잡고 자동으로 다음 동작 이어가도록 추가.</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -2423,7 +2457,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
@@ -2491,9 +2525,6 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1" indent="2"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="2"/>
-    </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1" indent="2"/>
     </xf>
@@ -2511,36 +2542,6 @@
     </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="3" fillId="4" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="3" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="3" fillId="4" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="9" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2574,6 +2575,45 @@
     </xf>
     <xf numFmtId="49" fontId="8" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="3" fillId="4" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="3" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="3" fillId="4" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="2"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2865,12 +2905,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B2" s="34" t="s">
+      <c r="B2" s="44" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
+      <c r="C2" s="44"/>
+      <c r="D2" s="44"/>
+      <c r="E2" s="44"/>
     </row>
     <row r="3" spans="2:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="4" spans="2:8" s="3" customFormat="1" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2888,12 +2928,12 @@
       </c>
     </row>
     <row r="5" spans="2:8" s="3" customFormat="1" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="35" t="s">
+      <c r="B5" s="45" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="36"/>
-      <c r="D5" s="36"/>
-      <c r="E5" s="37"/>
+      <c r="C5" s="46"/>
+      <c r="D5" s="46"/>
+      <c r="E5" s="47"/>
     </row>
     <row r="6" spans="2:8" s="3" customFormat="1" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B6" s="13" t="s">
@@ -2967,12 +3007,12 @@
       <c r="H13" s="12"/>
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B16" s="34" t="s">
+      <c r="B16" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="C16" s="34"/>
-      <c r="D16" s="34"/>
-      <c r="E16" s="34"/>
+      <c r="C16" s="44"/>
+      <c r="D16" s="44"/>
+      <c r="E16" s="44"/>
     </row>
     <row r="17" spans="2:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="18" spans="2:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -3035,13 +3075,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B66418C2-2F25-4DF5-AD93-3985FBAF3208}">
-  <dimension ref="B1:D101"/>
+  <dimension ref="B1:D105"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
     <col min="2" max="2" width="9.875" style="20" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="102.375" style="23" customWidth="1"/>
-    <col min="4" max="4" width="72.375" style="8" customWidth="1"/>
+    <col min="3" max="3" width="92.25" style="23" customWidth="1"/>
+    <col min="4" max="4" width="76.25" style="8" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:4" ht="9.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
@@ -3057,17 +3097,17 @@
       </c>
     </row>
     <row r="3" spans="2:4" ht="25.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="41" t="s">
+      <c r="B3" s="51" t="s">
         <v>620</v>
       </c>
-      <c r="C3" s="42"/>
-      <c r="D3" s="43"/>
+      <c r="C3" s="52"/>
+      <c r="D3" s="53"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B4" s="18" t="s">
         <v>617</v>
       </c>
-      <c r="C4" s="49" t="s">
+      <c r="C4" s="38" t="s">
         <v>621</v>
       </c>
       <c r="D4" s="10"/>
@@ -3076,7 +3116,7 @@
       <c r="B5" s="18" t="s">
         <v>617</v>
       </c>
-      <c r="C5" s="50" t="s">
+      <c r="C5" s="39" t="s">
         <v>622</v>
       </c>
       <c r="D5" s="10"/>
@@ -3085,7 +3125,7 @@
       <c r="B6" s="18" t="s">
         <v>617</v>
       </c>
-      <c r="C6" s="51" t="s">
+      <c r="C6" s="40" t="s">
         <v>623</v>
       </c>
       <c r="D6" s="15"/>
@@ -3094,7 +3134,7 @@
       <c r="B7" s="18" t="s">
         <v>624</v>
       </c>
-      <c r="C7" s="52" t="s">
+      <c r="C7" s="41" t="s">
         <v>625</v>
       </c>
       <c r="D7" s="15"/>
@@ -3103,7 +3143,7 @@
       <c r="B8" s="18" t="s">
         <v>626</v>
       </c>
-      <c r="C8" s="51" t="s">
+      <c r="C8" s="40" t="s">
         <v>627</v>
       </c>
       <c r="D8" s="15"/>
@@ -3112,7 +3152,7 @@
       <c r="B9" s="18" t="s">
         <v>629</v>
       </c>
-      <c r="C9" s="51" t="s">
+      <c r="C9" s="40" t="s">
         <v>628</v>
       </c>
       <c r="D9" s="10"/>
@@ -3121,7 +3161,7 @@
       <c r="B10" s="18" t="s">
         <v>630</v>
       </c>
-      <c r="C10" s="51" t="s">
+      <c r="C10" s="40" t="s">
         <v>631</v>
       </c>
       <c r="D10" s="16"/>
@@ -3130,7 +3170,7 @@
       <c r="B11" s="18" t="s">
         <v>632</v>
       </c>
-      <c r="C11" s="51" t="s">
+      <c r="C11" s="40" t="s">
         <v>633</v>
       </c>
       <c r="D11" s="15"/>
@@ -3139,14 +3179,14 @@
       <c r="B12" s="18" t="s">
         <v>634</v>
       </c>
-      <c r="C12" s="51" t="s">
+      <c r="C12" s="40" t="s">
         <v>635</v>
       </c>
       <c r="D12" s="15"/>
     </row>
     <row r="13" spans="2:4" ht="26.25" x14ac:dyDescent="0.3">
       <c r="B13" s="18"/>
-      <c r="C13" s="44" t="s">
+      <c r="C13" s="33" t="s">
         <v>637</v>
       </c>
       <c r="D13" s="10"/>
@@ -3155,7 +3195,7 @@
       <c r="B14" s="18" t="s">
         <v>636</v>
       </c>
-      <c r="C14" s="53" t="s">
+      <c r="C14" s="42" t="s">
         <v>638</v>
       </c>
       <c r="D14" s="10"/>
@@ -3164,7 +3204,7 @@
       <c r="B15" s="18" t="s">
         <v>636</v>
       </c>
-      <c r="C15" s="53" t="s">
+      <c r="C15" s="42" t="s">
         <v>639</v>
       </c>
       <c r="D15" s="10"/>
@@ -3173,7 +3213,7 @@
       <c r="B16" s="18" t="s">
         <v>636</v>
       </c>
-      <c r="C16" s="53" t="s">
+      <c r="C16" s="42" t="s">
         <v>640</v>
       </c>
       <c r="D16" s="10"/>
@@ -3182,7 +3222,7 @@
       <c r="B17" s="18" t="s">
         <v>636</v>
       </c>
-      <c r="C17" s="54" t="s">
+      <c r="C17" s="43" t="s">
         <v>642</v>
       </c>
       <c r="D17" s="10"/>
@@ -3191,7 +3231,7 @@
       <c r="B18" s="18" t="s">
         <v>636</v>
       </c>
-      <c r="C18" s="53" t="s">
+      <c r="C18" s="42" t="s">
         <v>641</v>
       </c>
       <c r="D18" s="10"/>
@@ -3200,152 +3240,180 @@
       <c r="B19" s="18" t="s">
         <v>636</v>
       </c>
-      <c r="C19" s="53" t="s">
+      <c r="C19" s="42" t="s">
         <v>643</v>
       </c>
       <c r="D19" s="10"/>
     </row>
-    <row r="20" spans="2:4" s="47" customFormat="1" ht="148.5" x14ac:dyDescent="0.3">
-      <c r="B20" s="45" t="s">
+    <row r="20" spans="2:4" s="36" customFormat="1" ht="148.5" x14ac:dyDescent="0.3">
+      <c r="B20" s="34" t="s">
         <v>636</v>
       </c>
-      <c r="C20" s="48" t="s">
+      <c r="C20" s="37" t="s">
         <v>644</v>
       </c>
-      <c r="D20" s="46" t="s">
+      <c r="D20" s="35" t="s">
         <v>645</v>
       </c>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B21" s="18"/>
-      <c r="C21" s="27"/>
+      <c r="B21" s="18" t="s">
+        <v>652</v>
+      </c>
+      <c r="C21" s="54" t="s">
+        <v>646</v>
+      </c>
       <c r="D21" s="10"/>
     </row>
     <row r="22" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B22" s="18"/>
-      <c r="C22" s="28"/>
+      <c r="B22" s="18" t="s">
+        <v>652</v>
+      </c>
+      <c r="C22" s="55" t="s">
+        <v>647</v>
+      </c>
       <c r="D22" s="10"/>
     </row>
     <row r="23" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B23" s="18"/>
-      <c r="C23" s="28"/>
+      <c r="B23" s="18" t="s">
+        <v>652</v>
+      </c>
+      <c r="C23" s="55" t="s">
+        <v>648</v>
+      </c>
       <c r="D23" s="10"/>
     </row>
     <row r="24" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B24" s="18"/>
-      <c r="C24" s="28"/>
+      <c r="B24" s="18" t="s">
+        <v>651</v>
+      </c>
+      <c r="C24" s="55" t="s">
+        <v>649</v>
+      </c>
       <c r="D24" s="10"/>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B25" s="18"/>
-      <c r="C25" s="28"/>
+      <c r="B25" s="18" t="s">
+        <v>651</v>
+      </c>
+      <c r="C25" s="55" t="s">
+        <v>650</v>
+      </c>
       <c r="D25" s="10"/>
     </row>
     <row r="26" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B26" s="18"/>
-      <c r="C26" s="28"/>
+      <c r="B26" s="18" t="s">
+        <v>651</v>
+      </c>
+      <c r="C26" s="56" t="s">
+        <v>653</v>
+      </c>
       <c r="D26" s="10"/>
     </row>
     <row r="27" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B27" s="18"/>
-      <c r="C27" s="29"/>
+      <c r="B27" s="18" t="s">
+        <v>652</v>
+      </c>
+      <c r="C27" s="56" t="s">
+        <v>654</v>
+      </c>
       <c r="D27" s="10"/>
     </row>
     <row r="28" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B28" s="18"/>
-      <c r="C28" s="29"/>
+      <c r="C28" s="56"/>
       <c r="D28" s="10"/>
     </row>
     <row r="29" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B29" s="18"/>
-      <c r="C29" s="29"/>
+      <c r="C29" s="56"/>
       <c r="D29" s="10"/>
     </row>
     <row r="30" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B30" s="18"/>
-      <c r="C30" s="28"/>
+      <c r="C30" s="56"/>
       <c r="D30" s="10"/>
     </row>
-    <row r="31" spans="2:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B31" s="18"/>
-      <c r="C31" s="30"/>
+      <c r="C31" s="28"/>
       <c r="D31" s="10"/>
     </row>
-    <row r="32" spans="2:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B32" s="38" t="s">
-        <v>619</v>
-      </c>
-      <c r="C32" s="39"/>
-      <c r="D32" s="40"/>
+    <row r="32" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B32" s="18"/>
+      <c r="C32" s="28"/>
+      <c r="D32" s="10"/>
     </row>
     <row r="33" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B33" s="18"/>
-      <c r="C33" s="31"/>
+      <c r="C33" s="28"/>
       <c r="D33" s="10"/>
     </row>
     <row r="34" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B34" s="18"/>
-      <c r="C34" s="32"/>
+      <c r="C34" s="27"/>
       <c r="D34" s="10"/>
     </row>
-    <row r="35" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B35" s="18"/>
-      <c r="C35" s="31"/>
+      <c r="C35" s="29"/>
       <c r="D35" s="10"/>
     </row>
-    <row r="36" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B36" s="18"/>
-      <c r="C36" s="32"/>
-      <c r="D36" s="10"/>
+    <row r="36" spans="2:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B36" s="48" t="s">
+        <v>619</v>
+      </c>
+      <c r="C36" s="49"/>
+      <c r="D36" s="50"/>
     </row>
     <row r="37" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B37" s="18"/>
-      <c r="C37" s="32"/>
+      <c r="C37" s="30"/>
       <c r="D37" s="10"/>
     </row>
     <row r="38" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B38" s="18"/>
-      <c r="C38" s="32"/>
+      <c r="C38" s="31"/>
       <c r="D38" s="10"/>
     </row>
     <row r="39" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B39" s="18"/>
-      <c r="C39" s="32"/>
+      <c r="C39" s="30"/>
       <c r="D39" s="10"/>
     </row>
     <row r="40" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B40" s="18"/>
-      <c r="C40" s="32"/>
+      <c r="C40" s="31"/>
       <c r="D40" s="10"/>
     </row>
     <row r="41" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B41" s="18"/>
-      <c r="C41" s="32"/>
+      <c r="C41" s="31"/>
       <c r="D41" s="10"/>
     </row>
     <row r="42" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B42" s="18"/>
-      <c r="C42" s="32"/>
+      <c r="C42" s="31"/>
       <c r="D42" s="10"/>
     </row>
     <row r="43" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B43" s="18"/>
-      <c r="C43" s="32"/>
+      <c r="C43" s="31"/>
       <c r="D43" s="10"/>
     </row>
     <row r="44" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B44" s="18"/>
-      <c r="C44" s="32"/>
+      <c r="C44" s="31"/>
       <c r="D44" s="10"/>
     </row>
     <row r="45" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B45" s="18"/>
-      <c r="C45" s="32"/>
+      <c r="C45" s="31"/>
       <c r="D45" s="10"/>
     </row>
     <row r="46" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B46" s="18"/>
-      <c r="C46" s="32"/>
+      <c r="C46" s="31"/>
       <c r="D46" s="10"/>
     </row>
     <row r="47" spans="2:4" x14ac:dyDescent="0.3">
@@ -3365,77 +3433,77 @@
     </row>
     <row r="50" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B50" s="18"/>
-      <c r="C50" s="32"/>
+      <c r="C50" s="31"/>
       <c r="D50" s="10"/>
     </row>
     <row r="51" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B51" s="18"/>
-      <c r="C51" s="32"/>
+      <c r="C51" s="30"/>
       <c r="D51" s="10"/>
     </row>
     <row r="52" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B52" s="18"/>
-      <c r="C52" s="31"/>
+      <c r="C52" s="30"/>
       <c r="D52" s="10"/>
     </row>
     <row r="53" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B53" s="18"/>
-      <c r="C53" s="32"/>
+      <c r="C53" s="30"/>
       <c r="D53" s="10"/>
     </row>
     <row r="54" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B54" s="18"/>
-      <c r="C54" s="29"/>
+      <c r="C54" s="31"/>
       <c r="D54" s="10"/>
     </row>
     <row r="55" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B55" s="18"/>
-      <c r="C55" s="29"/>
+      <c r="C55" s="31"/>
       <c r="D55" s="10"/>
     </row>
     <row r="56" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B56" s="18"/>
-      <c r="C56" s="32"/>
+      <c r="C56" s="30"/>
       <c r="D56" s="10"/>
     </row>
     <row r="57" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B57" s="18"/>
-      <c r="C57" s="32"/>
+      <c r="C57" s="31"/>
       <c r="D57" s="10"/>
     </row>
     <row r="58" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B58" s="18"/>
-      <c r="C58" s="32"/>
+      <c r="C58" s="28"/>
       <c r="D58" s="10"/>
     </row>
     <row r="59" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B59" s="18"/>
-      <c r="C59" s="32"/>
+      <c r="C59" s="28"/>
       <c r="D59" s="10"/>
     </row>
     <row r="60" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B60" s="18"/>
-      <c r="C60" s="32"/>
+      <c r="C60" s="31"/>
       <c r="D60" s="10"/>
     </row>
     <row r="61" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B61" s="18"/>
-      <c r="C61" s="32"/>
+      <c r="C61" s="31"/>
       <c r="D61" s="10"/>
     </row>
     <row r="62" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B62" s="18"/>
-      <c r="C62" s="32"/>
+      <c r="C62" s="31"/>
       <c r="D62" s="10"/>
     </row>
     <row r="63" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B63" s="18"/>
-      <c r="C63" s="29"/>
+      <c r="C63" s="31"/>
       <c r="D63" s="10"/>
     </row>
     <row r="64" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B64" s="18"/>
-      <c r="C64" s="32"/>
+      <c r="C64" s="31"/>
       <c r="D64" s="10"/>
     </row>
     <row r="65" spans="2:4" x14ac:dyDescent="0.3">
@@ -3445,22 +3513,22 @@
     </row>
     <row r="66" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B66" s="18"/>
-      <c r="C66" s="29"/>
+      <c r="C66" s="31"/>
       <c r="D66" s="10"/>
     </row>
     <row r="67" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B67" s="18"/>
-      <c r="C67" s="32"/>
+      <c r="C67" s="28"/>
       <c r="D67" s="10"/>
     </row>
     <row r="68" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B68" s="18"/>
-      <c r="C68" s="29"/>
+      <c r="C68" s="31"/>
       <c r="D68" s="10"/>
     </row>
     <row r="69" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B69" s="18"/>
-      <c r="C69" s="29"/>
+      <c r="C69" s="30"/>
       <c r="D69" s="10"/>
     </row>
     <row r="70" spans="2:4" x14ac:dyDescent="0.3">
@@ -3470,47 +3538,47 @@
     </row>
     <row r="71" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B71" s="18"/>
-      <c r="C71" s="26"/>
-      <c r="D71" s="17"/>
+      <c r="C71" s="31"/>
+      <c r="D71" s="10"/>
     </row>
     <row r="72" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B72" s="18"/>
-      <c r="C72" s="32"/>
+      <c r="C72" s="28"/>
       <c r="D72" s="10"/>
     </row>
     <row r="73" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B73" s="18"/>
-      <c r="C73" s="32"/>
+      <c r="C73" s="28"/>
       <c r="D73" s="10"/>
     </row>
     <row r="74" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B74" s="18"/>
-      <c r="C74" s="32"/>
+      <c r="C74" s="27"/>
       <c r="D74" s="10"/>
     </row>
     <row r="75" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B75" s="18"/>
-      <c r="C75" s="32"/>
-      <c r="D75" s="10"/>
+      <c r="C75" s="26"/>
+      <c r="D75" s="17"/>
     </row>
     <row r="76" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B76" s="18"/>
-      <c r="C76" s="32"/>
+      <c r="C76" s="31"/>
       <c r="D76" s="10"/>
     </row>
     <row r="77" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B77" s="18"/>
-      <c r="C77" s="26"/>
+      <c r="C77" s="31"/>
       <c r="D77" s="10"/>
     </row>
     <row r="78" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B78" s="18"/>
-      <c r="C78" s="32"/>
+      <c r="C78" s="31"/>
       <c r="D78" s="10"/>
     </row>
     <row r="79" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B79" s="18"/>
-      <c r="C79" s="26"/>
+      <c r="C79" s="31"/>
       <c r="D79" s="10"/>
     </row>
     <row r="80" spans="2:4" x14ac:dyDescent="0.3">
@@ -3520,12 +3588,12 @@
     </row>
     <row r="81" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B81" s="18"/>
-      <c r="C81" s="31"/>
+      <c r="C81" s="26"/>
       <c r="D81" s="10"/>
     </row>
     <row r="82" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B82" s="18"/>
-      <c r="C82" s="26"/>
+      <c r="C82" s="31"/>
       <c r="D82" s="10"/>
     </row>
     <row r="83" spans="2:4" x14ac:dyDescent="0.3">
@@ -3535,12 +3603,12 @@
     </row>
     <row r="84" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B84" s="18"/>
-      <c r="C84" s="26"/>
+      <c r="C84" s="30"/>
       <c r="D84" s="10"/>
     </row>
     <row r="85" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B85" s="18"/>
-      <c r="C85" s="26"/>
+      <c r="C85" s="30"/>
       <c r="D85" s="10"/>
     </row>
     <row r="86" spans="2:4" x14ac:dyDescent="0.3">
@@ -3575,37 +3643,37 @@
     </row>
     <row r="92" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B92" s="18"/>
-      <c r="C92" s="25"/>
+      <c r="C92" s="26"/>
       <c r="D92" s="10"/>
     </row>
     <row r="93" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B93" s="18"/>
-      <c r="C93" s="25"/>
+      <c r="C93" s="26"/>
       <c r="D93" s="10"/>
     </row>
     <row r="94" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B94" s="18"/>
-      <c r="C94" s="25"/>
+      <c r="C94" s="26"/>
       <c r="D94" s="10"/>
     </row>
     <row r="95" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B95" s="18"/>
-      <c r="C95" s="30"/>
+      <c r="C95" s="26"/>
       <c r="D95" s="10"/>
     </row>
     <row r="96" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B96" s="18"/>
-      <c r="C96" s="30"/>
+      <c r="C96" s="25"/>
       <c r="D96" s="10"/>
     </row>
     <row r="97" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B97" s="18"/>
-      <c r="C97" s="30"/>
+      <c r="C97" s="25"/>
       <c r="D97" s="10"/>
     </row>
     <row r="98" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B98" s="18"/>
-      <c r="C98" s="30"/>
+      <c r="C98" s="25"/>
       <c r="D98" s="10"/>
     </row>
     <row r="99" spans="2:4" x14ac:dyDescent="0.3">
@@ -3618,14 +3686,34 @@
       <c r="C100" s="29"/>
       <c r="D100" s="10"/>
     </row>
-    <row r="101" spans="2:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B101" s="22"/>
-      <c r="C101" s="33"/>
-      <c r="D101" s="11"/>
+    <row r="101" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B101" s="18"/>
+      <c r="C101" s="29"/>
+      <c r="D101" s="10"/>
+    </row>
+    <row r="102" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B102" s="18"/>
+      <c r="C102" s="29"/>
+      <c r="D102" s="10"/>
+    </row>
+    <row r="103" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B103" s="18"/>
+      <c r="C103" s="28"/>
+      <c r="D103" s="10"/>
+    </row>
+    <row r="104" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B104" s="18"/>
+      <c r="C104" s="28"/>
+      <c r="D104" s="10"/>
+    </row>
+    <row r="105" spans="2:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B105" s="22"/>
+      <c r="C105" s="32"/>
+      <c r="D105" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="B36:D36"/>
     <mergeCell ref="B3:D3"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>

<commit_message>
2026 09 15 003
servo moving 판넬 수정.
</commit_message>
<xml_diff>
--- a/.IBC_인도 NGSORTER 셋업(2026 06).xlsx
+++ b/.IBC_인도 NGSORTER 셋업(2026 06).xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84F46ADC-6439-4E8B-9FE6-4BADAA0F02B7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEBC9C13-E693-4C38-90B8-B0BCE557F83A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="8910" windowHeight="10470" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="670" uniqueCount="655">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="672" uniqueCount="657">
   <si>
     <t>내용</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -2115,11 +2115,19 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>불량선별기 PLC 비상정지 버튼 눌렀을때 서보 멈춤. 에러표시 (pause, 알람)</t>
+    <t>비상정지시 셀을 들고 있는 상태에서 홈잡고 자동으로 다음 동작 이어가도록 추가.</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>비상정지시 셀을 들고 있는 상태에서 홈잡고 자동으로 다음 동작 이어가도록 추가.</t>
+    <t>불량선별기 PLC 비상정지 버튼 눌렀을때 서보 멈춤. 에러표시 (pause, 알람) =&gt; 차후</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>9/15</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>수동작업 완료버튼 테스트.</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -2131,7 +2139,7 @@
     <numFmt numFmtId="176" formatCode="mm&quot;월&quot;\ dd&quot;일&quot;"/>
     <numFmt numFmtId="177" formatCode="&quot;₩&quot;#,##0"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2209,6 +2217,15 @@
     <font>
       <b/>
       <sz val="16"/>
+      <color rgb="FFFF0000"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="맑은 고딕"/>
       <family val="3"/>
@@ -2457,7 +2474,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
@@ -2576,6 +2593,15 @@
     <xf numFmtId="49" fontId="8" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="2"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2606,13 +2632,7 @@
     <xf numFmtId="176" fontId="3" fillId="4" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="2"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="2"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1" indent="2"/>
     </xf>
   </cellXfs>
@@ -2905,12 +2925,12 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B2" s="44" t="s">
+      <c r="B2" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="44"/>
-      <c r="D2" s="44"/>
-      <c r="E2" s="44"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
     </row>
     <row r="3" spans="2:8" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="4" spans="2:8" s="3" customFormat="1" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -2928,12 +2948,12 @@
       </c>
     </row>
     <row r="5" spans="2:8" s="3" customFormat="1" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="45" t="s">
+      <c r="B5" s="48" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="46"/>
-      <c r="D5" s="46"/>
-      <c r="E5" s="47"/>
+      <c r="C5" s="49"/>
+      <c r="D5" s="49"/>
+      <c r="E5" s="50"/>
     </row>
     <row r="6" spans="2:8" s="3" customFormat="1" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B6" s="13" t="s">
@@ -3007,12 +3027,12 @@
       <c r="H13" s="12"/>
     </row>
     <row r="16" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B16" s="44" t="s">
+      <c r="B16" s="47" t="s">
         <v>14</v>
       </c>
-      <c r="C16" s="44"/>
-      <c r="D16" s="44"/>
-      <c r="E16" s="44"/>
+      <c r="C16" s="47"/>
+      <c r="D16" s="47"/>
+      <c r="E16" s="47"/>
     </row>
     <row r="17" spans="2:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="18" spans="2:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
@@ -3097,11 +3117,11 @@
       </c>
     </row>
     <row r="3" spans="2:4" ht="25.5" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="51" t="s">
+      <c r="B3" s="54" t="s">
         <v>620</v>
       </c>
-      <c r="C3" s="52"/>
-      <c r="D3" s="53"/>
+      <c r="C3" s="55"/>
+      <c r="D3" s="56"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B4" s="18" t="s">
@@ -3240,7 +3260,7 @@
       <c r="B19" s="18" t="s">
         <v>636</v>
       </c>
-      <c r="C19" s="42" t="s">
+      <c r="C19" s="43" t="s">
         <v>643</v>
       </c>
       <c r="D19" s="10"/>
@@ -3260,7 +3280,7 @@
       <c r="B21" s="18" t="s">
         <v>652</v>
       </c>
-      <c r="C21" s="54" t="s">
+      <c r="C21" s="44" t="s">
         <v>646</v>
       </c>
       <c r="D21" s="10"/>
@@ -3269,7 +3289,7 @@
       <c r="B22" s="18" t="s">
         <v>652</v>
       </c>
-      <c r="C22" s="55" t="s">
+      <c r="C22" s="45" t="s">
         <v>647</v>
       </c>
       <c r="D22" s="10"/>
@@ -3278,7 +3298,7 @@
       <c r="B23" s="18" t="s">
         <v>652</v>
       </c>
-      <c r="C23" s="55" t="s">
+      <c r="C23" s="45" t="s">
         <v>648</v>
       </c>
       <c r="D23" s="10"/>
@@ -3287,7 +3307,7 @@
       <c r="B24" s="18" t="s">
         <v>651</v>
       </c>
-      <c r="C24" s="55" t="s">
+      <c r="C24" s="57" t="s">
         <v>649</v>
       </c>
       <c r="D24" s="10"/>
@@ -3296,7 +3316,7 @@
       <c r="B25" s="18" t="s">
         <v>651</v>
       </c>
-      <c r="C25" s="55" t="s">
+      <c r="C25" s="45" t="s">
         <v>650</v>
       </c>
       <c r="D25" s="10"/>
@@ -3305,8 +3325,8 @@
       <c r="B26" s="18" t="s">
         <v>651</v>
       </c>
-      <c r="C26" s="56" t="s">
-        <v>653</v>
+      <c r="C26" s="46" t="s">
+        <v>654</v>
       </c>
       <c r="D26" s="10"/>
     </row>
@@ -3314,24 +3334,28 @@
       <c r="B27" s="18" t="s">
         <v>652</v>
       </c>
-      <c r="C27" s="56" t="s">
-        <v>654</v>
+      <c r="C27" s="46" t="s">
+        <v>653</v>
       </c>
       <c r="D27" s="10"/>
     </row>
     <row r="28" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B28" s="18"/>
-      <c r="C28" s="56"/>
+      <c r="B28" s="18" t="s">
+        <v>655</v>
+      </c>
+      <c r="C28" s="46" t="s">
+        <v>656</v>
+      </c>
       <c r="D28" s="10"/>
     </row>
     <row r="29" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B29" s="18"/>
-      <c r="C29" s="56"/>
+      <c r="C29" s="46"/>
       <c r="D29" s="10"/>
     </row>
     <row r="30" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B30" s="18"/>
-      <c r="C30" s="56"/>
+      <c r="C30" s="46"/>
       <c r="D30" s="10"/>
     </row>
     <row r="31" spans="2:4" x14ac:dyDescent="0.3">
@@ -3360,11 +3384,11 @@
       <c r="D35" s="10"/>
     </row>
     <row r="36" spans="2:4" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B36" s="48" t="s">
+      <c r="B36" s="51" t="s">
         <v>619</v>
       </c>
-      <c r="C36" s="49"/>
-      <c r="D36" s="50"/>
+      <c r="C36" s="52"/>
+      <c r="D36" s="53"/>
     </row>
     <row r="37" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B37" s="18"/>

</xml_diff>